<commit_message>
MAJ liste activites avec donnees reelles Sprint 1
</commit_message>
<xml_diff>
--- a/docs/TP2-FoxTrot-Liste_Activites-H26.xlsx
+++ b/docs/TP2-FoxTrot-Liste_Activites-H26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UQAM\Été 2026\INF6150 (Génie logiciel - Conduite de projets informatiques)\Travaux Pratiques\TP2\fixmycar\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51BC895F-2152-49FA-83C0-8AA9A6B3D0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC39A44-B1DA-46CA-BF0A-825A7C3568EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Activités" sheetId="1" r:id="rId1"/>
@@ -3439,11 +3439,11 @@
       </c>
       <c r="AF11" s="156">
         <f>U37</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="AG11" s="162">
         <f>Z37</f>
-        <v>0</v>
+        <v>1430</v>
       </c>
       <c r="AH11" s="157">
         <v>9</v>
@@ -3604,11 +3604,11 @@
       </c>
       <c r="AF13" s="168">
         <f>U45</f>
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="AG13" s="169">
         <f>Z45</f>
-        <v>7480</v>
+        <v>8910</v>
       </c>
       <c r="AH13" s="170">
         <v>2</v>
@@ -3713,11 +3713,11 @@
       </c>
       <c r="AF14" s="154">
         <f>V45</f>
-        <v>270</v>
+        <v>257</v>
       </c>
       <c r="AG14" s="161">
         <f>V45*tarif</f>
-        <v>29700</v>
+        <v>28270</v>
       </c>
       <c r="AH14" s="153">
         <v>7</v>
@@ -4154,31 +4154,43 @@
         <v>1430</v>
       </c>
       <c r="L19" s="9"/>
-      <c r="M19" s="106"/>
+      <c r="M19" s="106">
+        <v>46212</v>
+      </c>
       <c r="N19" s="136">
         <f t="shared" ref="N19:N36" si="27">M19-C19</f>
-        <v>-46194</v>
+        <v>18</v>
       </c>
       <c r="O19" s="121"/>
-      <c r="P19" s="131"/>
-      <c r="Q19" s="131"/>
-      <c r="R19" s="131"/>
-      <c r="S19" s="131"/>
-      <c r="T19" s="131"/>
+      <c r="P19" s="131">
+        <v>8</v>
+      </c>
+      <c r="Q19" s="131">
+        <v>1</v>
+      </c>
+      <c r="R19" s="131">
+        <v>1</v>
+      </c>
+      <c r="S19" s="131">
+        <v>1</v>
+      </c>
+      <c r="T19" s="131">
+        <v>2</v>
+      </c>
       <c r="U19" s="137">
         <f t="shared" ref="U19:U36" si="28">SUM(P19:T19)</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="V19" s="131">
         <f>J19-U19</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="W19" s="137">
         <f t="shared" ref="W19:W36" si="29">U19+V19</f>
         <v>13</v>
       </c>
       <c r="X19" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y19" s="137">
         <f t="shared" ref="Y19:Y36" si="30">(W19-J19)</f>
@@ -4186,7 +4198,7 @@
       </c>
       <c r="Z19" s="109">
         <f t="shared" ref="Z19:Z36" si="31">tarif*U19</f>
-        <v>0</v>
+        <v>1430</v>
       </c>
       <c r="AA19" s="109">
         <f t="shared" ref="AA19:AA37" si="32">tarif*W19</f>
@@ -4194,7 +4206,7 @@
       </c>
       <c r="AB19" s="139">
         <f t="shared" ref="AB19:AB37" si="33">Z19-K19</f>
-        <v>-1430</v>
+        <v>0</v>
       </c>
       <c r="AC19" s="6"/>
       <c r="AE19" s="203"/>
@@ -5694,11 +5706,11 @@
       <c r="L37" s="49"/>
       <c r="M37" s="46">
         <f>MAX(M19:M36)</f>
-        <v>0</v>
+        <v>46212</v>
       </c>
       <c r="N37" s="48">
         <f>M37-C37</f>
-        <v>-46236</v>
+        <v>-24</v>
       </c>
       <c r="O37" s="47">
         <f>SUM(O21:O23)</f>
@@ -5706,31 +5718,31 @@
       </c>
       <c r="P37" s="48">
         <f t="shared" ref="P37:Y37" si="37">SUM(P19:P19)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q37" s="48">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R37" s="48">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S37" s="48">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T37" s="48">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U37" s="48">
         <f>SUM(U19:U36)</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="V37" s="48">
         <f>SUM(V19:V36)</f>
-        <v>230</v>
+        <v>217</v>
       </c>
       <c r="W37" s="48">
         <f>SUM(W19:W36)</f>
@@ -5743,7 +5755,7 @@
       </c>
       <c r="Z37" s="70">
         <f t="shared" ref="Z37" si="38">tarif*U37</f>
-        <v>0</v>
+        <v>1430</v>
       </c>
       <c r="AA37" s="70">
         <f t="shared" si="32"/>
@@ -5751,7 +5763,7 @@
       </c>
       <c r="AB37" s="70">
         <f t="shared" si="33"/>
-        <v>-25300</v>
+        <v>-23870</v>
       </c>
       <c r="AC37" s="50"/>
       <c r="AD37" s="37"/>
@@ -6354,11 +6366,11 @@
       <c r="L45" s="27"/>
       <c r="M45" s="64">
         <f>MAX(M11,M17,M37,M43)</f>
-        <v>46188</v>
+        <v>46212</v>
       </c>
       <c r="N45" s="65">
         <f>M45-C45</f>
-        <v>-55</v>
+        <v>-31</v>
       </c>
       <c r="O45" s="26">
         <f>O37</f>
@@ -6366,31 +6378,31 @@
       </c>
       <c r="P45" s="58">
         <f t="shared" ref="P45:W45" si="51">P11+P17+P37+P43</f>
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="Q45" s="58">
         <f t="shared" si="51"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R45" s="58">
         <f t="shared" si="51"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S45" s="58">
         <f t="shared" si="51"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T45" s="58">
         <f t="shared" si="51"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="U45" s="58">
         <f t="shared" si="51"/>
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="V45" s="58">
         <f t="shared" si="51"/>
-        <v>270</v>
+        <v>257</v>
       </c>
       <c r="W45" s="58">
         <f t="shared" si="51"/>
@@ -6403,7 +6415,7 @@
       </c>
       <c r="Z45" s="73">
         <f>Z11+Z17+Z37+Z43</f>
-        <v>7480</v>
+        <v>8910</v>
       </c>
       <c r="AA45" s="73">
         <f>AA11+AA17+AA37+AA43</f>
@@ -6411,7 +6423,7 @@
       </c>
       <c r="AB45" s="73">
         <f>Z45-K45</f>
-        <v>-29700</v>
+        <v>-28270</v>
       </c>
       <c r="AC45" s="63"/>
       <c r="AD45" s="28"/>

</xml_diff>